<commit_message>
Engine v2: assumptions, redirects, trail, timeline, scenarios, tests (work in progress)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fixtures/applications.xlsx
+++ b/fixtures/applications.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="154">
   <si>
     <t>Applications — one row per record. Row 3 is an example (grey); enter data from row 4.</t>
   </si>
@@ -162,9 +162,6 @@
     <t>Mangaluru</t>
   </si>
   <si>
-    <t>575002.0</t>
-  </si>
-  <si>
     <t>Mobile accessories shop</t>
   </si>
   <si>
@@ -222,6 +219,9 @@
     <t>Latha Murthy</t>
   </si>
   <si>
+    <t>560010.0</t>
+  </si>
+  <si>
     <t>General store</t>
   </si>
   <si>
@@ -306,6 +306,54 @@
     <t>Irfan Pasha</t>
   </si>
   <si>
+    <t>APP-021</t>
+  </si>
+  <si>
+    <t>Prakash Joshi</t>
+  </si>
+  <si>
+    <t>Pune</t>
+  </si>
+  <si>
+    <t>Maharashtra</t>
+  </si>
+  <si>
+    <t>APP-022</t>
+  </si>
+  <si>
+    <t>Chitra Murthy</t>
+  </si>
+  <si>
+    <t>APP-023</t>
+  </si>
+  <si>
+    <t>Manjula Reddy</t>
+  </si>
+  <si>
+    <t>kannada &amp; english</t>
+  </si>
+  <si>
+    <t>APP-024</t>
+  </si>
+  <si>
+    <t>Naveen Reddy</t>
+  </si>
+  <si>
+    <t>ಕನ್ನಡ</t>
+  </si>
+  <si>
+    <t>APP-025</t>
+  </si>
+  <si>
+    <t>Savitha Rao</t>
+  </si>
+  <si>
+    <t>575003.0</t>
+  </si>
+  <si>
+    <t>Cloth store</t>
+  </si>
+  <si>
     <t>Territories — one row per record.</t>
   </si>
   <si>
@@ -339,7 +387,7 @@
     <t>TER-02</t>
   </si>
   <si>
-    <t>570001, 570002, 570004, 570008, 570009</t>
+    <t>570004, 570009, 570020</t>
   </si>
   <si>
     <t>TER-03</t>
@@ -803,7 +851,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N22"/>
+  <dimension ref="A1:N27"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -1132,8 +1180,8 @@
       <c r="D9" t="s">
         <v>18</v>
       </c>
-      <c r="E9" t="s">
-        <v>49</v>
+      <c r="E9">
+        <v>575002</v>
       </c>
       <c r="F9">
         <v>22</v>
@@ -1142,7 +1190,7 @@
         <v>1</v>
       </c>
       <c r="H9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I9" t="s">
         <v>20</v>
@@ -1151,7 +1199,7 @@
         <v>300</v>
       </c>
       <c r="K9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="L9">
         <v>3</v>
@@ -1160,18 +1208,18 @@
         <v>22</v>
       </c>
       <c r="N9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>52</v>
+      </c>
+      <c r="B10" t="s">
         <v>53</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>54</v>
-      </c>
-      <c r="C10" t="s">
-        <v>55</v>
       </c>
       <c r="D10" t="s">
         <v>18</v>
@@ -1186,7 +1234,7 @@
         <v>4</v>
       </c>
       <c r="H10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I10" t="s">
         <v>20</v>
@@ -1209,13 +1257,13 @@
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B11" t="s">
         <v>57</v>
       </c>
-      <c r="B11" t="s">
-        <v>58</v>
-      </c>
       <c r="C11" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D11" t="s">
         <v>18</v>
@@ -1230,7 +1278,7 @@
         <v>7</v>
       </c>
       <c r="H11" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I11" t="s">
         <v>20</v>
@@ -1253,13 +1301,13 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>59</v>
+      </c>
+      <c r="B12" t="s">
         <v>60</v>
       </c>
-      <c r="B12" t="s">
-        <v>61</v>
-      </c>
       <c r="C12" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D12" t="s">
         <v>18</v>
@@ -1274,7 +1322,7 @@
         <v>0</v>
       </c>
       <c r="H12" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I12" t="s">
         <v>20</v>
@@ -1292,18 +1340,18 @@
         <v>22</v>
       </c>
       <c r="N12" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>63</v>
+      </c>
+      <c r="B13" t="s">
         <v>64</v>
       </c>
-      <c r="B13" t="s">
-        <v>65</v>
-      </c>
       <c r="C13" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D13" t="s">
         <v>18</v>
@@ -1318,7 +1366,7 @@
         <v>3</v>
       </c>
       <c r="H13" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I13" t="s">
         <v>20</v>
@@ -1341,19 +1389,19 @@
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>66</v>
+      </c>
+      <c r="B14" t="s">
         <v>67</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C14" t="s">
+        <v>54</v>
+      </c>
+      <c r="D14" t="s">
+        <v>18</v>
+      </c>
+      <c r="E14" t="s">
         <v>68</v>
-      </c>
-      <c r="C14" t="s">
-        <v>55</v>
-      </c>
-      <c r="D14" t="s">
-        <v>18</v>
-      </c>
-      <c r="E14">
-        <v>560010</v>
       </c>
       <c r="F14">
         <v>36</v>
@@ -1655,7 +1703,7 @@
         <v>93</v>
       </c>
       <c r="C21" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D21" t="s">
         <v>18</v>
@@ -1732,6 +1780,226 @@
         <v>36</v>
       </c>
       <c r="N22" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>97</v>
+      </c>
+      <c r="B23" t="s">
+        <v>98</v>
+      </c>
+      <c r="C23" t="s">
+        <v>99</v>
+      </c>
+      <c r="D23" t="s">
+        <v>100</v>
+      </c>
+      <c r="E23">
+        <v>411001</v>
+      </c>
+      <c r="F23">
+        <v>40</v>
+      </c>
+      <c r="G23">
+        <v>6</v>
+      </c>
+      <c r="H23" t="s">
+        <v>19</v>
+      </c>
+      <c r="I23" t="s">
+        <v>26</v>
+      </c>
+      <c r="J23">
+        <v>600</v>
+      </c>
+      <c r="K23" t="s">
+        <v>21</v>
+      </c>
+      <c r="L23">
+        <v>3</v>
+      </c>
+      <c r="M23" t="s">
+        <v>36</v>
+      </c>
+      <c r="N23" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>101</v>
+      </c>
+      <c r="B24" t="s">
+        <v>102</v>
+      </c>
+      <c r="C24" t="s">
+        <v>17</v>
+      </c>
+      <c r="D24" t="s">
+        <v>18</v>
+      </c>
+      <c r="E24">
+        <v>570099</v>
+      </c>
+      <c r="F24">
+        <v>30</v>
+      </c>
+      <c r="G24">
+        <v>4</v>
+      </c>
+      <c r="H24" t="s">
+        <v>55</v>
+      </c>
+      <c r="I24" t="s">
+        <v>20</v>
+      </c>
+      <c r="J24">
+        <v>500</v>
+      </c>
+      <c r="K24" t="s">
+        <v>21</v>
+      </c>
+      <c r="L24">
+        <v>3</v>
+      </c>
+      <c r="M24" t="s">
+        <v>36</v>
+      </c>
+      <c r="N24" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>103</v>
+      </c>
+      <c r="B25" t="s">
+        <v>104</v>
+      </c>
+      <c r="C25" t="s">
+        <v>77</v>
+      </c>
+      <c r="D25" t="s">
+        <v>18</v>
+      </c>
+      <c r="E25">
+        <v>577001</v>
+      </c>
+      <c r="F25">
+        <v>18</v>
+      </c>
+      <c r="G25">
+        <v>2</v>
+      </c>
+      <c r="H25" t="s">
+        <v>69</v>
+      </c>
+      <c r="I25" t="s">
+        <v>20</v>
+      </c>
+      <c r="J25">
+        <v>450</v>
+      </c>
+      <c r="K25" t="s">
+        <v>21</v>
+      </c>
+      <c r="L25">
+        <v>4</v>
+      </c>
+      <c r="M25" t="s">
+        <v>105</v>
+      </c>
+      <c r="N25" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>106</v>
+      </c>
+      <c r="B26" t="s">
+        <v>107</v>
+      </c>
+      <c r="C26" t="s">
+        <v>77</v>
+      </c>
+      <c r="D26" t="s">
+        <v>18</v>
+      </c>
+      <c r="E26">
+        <v>577002</v>
+      </c>
+      <c r="F26">
+        <v>18</v>
+      </c>
+      <c r="G26">
+        <v>2</v>
+      </c>
+      <c r="H26" t="s">
+        <v>69</v>
+      </c>
+      <c r="I26" t="s">
+        <v>20</v>
+      </c>
+      <c r="J26">
+        <v>450</v>
+      </c>
+      <c r="K26" t="s">
+        <v>21</v>
+      </c>
+      <c r="L26">
+        <v>4</v>
+      </c>
+      <c r="M26" t="s">
+        <v>108</v>
+      </c>
+      <c r="N26" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>109</v>
+      </c>
+      <c r="B27" t="s">
+        <v>110</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27" t="s">
+        <v>18</v>
+      </c>
+      <c r="E27" t="s">
+        <v>111</v>
+      </c>
+      <c r="F27">
+        <v>25</v>
+      </c>
+      <c r="G27">
+        <v>1</v>
+      </c>
+      <c r="H27" t="s">
+        <v>112</v>
+      </c>
+      <c r="I27" t="s">
+        <v>20</v>
+      </c>
+      <c r="J27">
+        <v>450</v>
+      </c>
+      <c r="K27" t="s">
+        <v>21</v>
+      </c>
+      <c r="L27">
+        <v>4</v>
+      </c>
+      <c r="M27" t="s">
+        <v>36</v>
+      </c>
+      <c r="N27" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1748,12 +2016,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>97</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
@@ -1762,21 +2030,21 @@
         <v>4</v>
       </c>
       <c r="D2" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="E2" t="s">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="F2" t="s">
-        <v>101</v>
+        <v>117</v>
       </c>
       <c r="G2" t="s">
-        <v>102</v>
+        <v>118</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>103</v>
+        <v>119</v>
       </c>
       <c r="B3" t="s">
         <v>17</v>
@@ -1785,21 +2053,21 @@
         <v>18</v>
       </c>
       <c r="D3" t="s">
-        <v>104</v>
+        <v>120</v>
       </c>
       <c r="E3" t="s">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="F3">
         <v>3</v>
       </c>
       <c r="G3" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="B4" t="s">
         <v>17</v>
@@ -1808,44 +2076,44 @@
         <v>18</v>
       </c>
       <c r="D4" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="E4" t="s">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="F4">
         <v>2</v>
       </c>
       <c r="G4" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>109</v>
+        <v>125</v>
       </c>
       <c r="B5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C5" t="s">
         <v>18</v>
       </c>
       <c r="D5" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="E5" t="s">
-        <v>111</v>
+        <v>127</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G5" t="s">
-        <v>112</v>
+        <v>128</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>113</v>
+        <v>129</v>
       </c>
       <c r="B6" t="s">
         <v>48</v>
@@ -1854,21 +2122,21 @@
         <v>18</v>
       </c>
       <c r="D6" t="s">
-        <v>114</v>
+        <v>130</v>
       </c>
       <c r="E6" t="s">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="F6">
         <v>1</v>
       </c>
       <c r="G6" t="s">
-        <v>115</v>
+        <v>131</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>116</v>
+        <v>132</v>
       </c>
       <c r="B7" t="s">
         <v>73</v>
@@ -1877,21 +2145,21 @@
         <v>18</v>
       </c>
       <c r="D7" t="s">
-        <v>117</v>
+        <v>133</v>
       </c>
       <c r="E7" t="s">
-        <v>118</v>
+        <v>134</v>
       </c>
       <c r="F7">
         <v>1</v>
       </c>
       <c r="G7" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>119</v>
+        <v>135</v>
       </c>
       <c r="B8" t="s">
         <v>77</v>
@@ -1900,21 +2168,21 @@
         <v>18</v>
       </c>
       <c r="D8" t="s">
-        <v>120</v>
+        <v>136</v>
       </c>
       <c r="E8" t="s">
-        <v>118</v>
+        <v>134</v>
       </c>
       <c r="F8">
         <v>1</v>
       </c>
       <c r="G8" t="s">
-        <v>112</v>
+        <v>128</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>121</v>
+        <v>137</v>
       </c>
       <c r="B9" t="s">
         <v>81</v>
@@ -1923,21 +2191,21 @@
         <v>18</v>
       </c>
       <c r="D9" t="s">
-        <v>122</v>
+        <v>138</v>
       </c>
       <c r="E9" t="s">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="F9">
         <v>2</v>
       </c>
       <c r="G9" t="s">
-        <v>112</v>
+        <v>128</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>123</v>
+        <v>139</v>
       </c>
       <c r="B10" t="s">
         <v>88</v>
@@ -1946,16 +2214,16 @@
         <v>18</v>
       </c>
       <c r="D10" t="s">
-        <v>124</v>
+        <v>140</v>
       </c>
       <c r="E10" t="s">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="F10">
         <v>1</v>
       </c>
       <c r="G10" t="s">
-        <v>112</v>
+        <v>128</v>
       </c>
     </row>
   </sheetData>
@@ -1971,12 +2239,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>125</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>126</v>
+        <v>142</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
@@ -1985,15 +2253,15 @@
         <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>127</v>
+        <v>143</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>128</v>
+        <v>144</v>
       </c>
       <c r="B3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C3">
         <v>560001</v>
@@ -2004,10 +2272,10 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>129</v>
+        <v>145</v>
       </c>
       <c r="B4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C4">
         <v>560034</v>
@@ -2018,10 +2286,10 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>130</v>
+        <v>146</v>
       </c>
       <c r="B5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C5">
         <v>560038</v>
@@ -2032,10 +2300,10 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>131</v>
+        <v>147</v>
       </c>
       <c r="B6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C6">
         <v>560066</v>
@@ -2046,10 +2314,10 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>132</v>
+        <v>148</v>
       </c>
       <c r="B7" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C7">
         <v>560076</v>
@@ -2060,7 +2328,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>133</v>
+        <v>149</v>
       </c>
       <c r="B8" t="s">
         <v>17</v>
@@ -2074,7 +2342,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="B9" t="s">
         <v>17</v>
@@ -2088,7 +2356,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>135</v>
+        <v>151</v>
       </c>
       <c r="B10" t="s">
         <v>48</v>
@@ -2102,7 +2370,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>136</v>
+        <v>152</v>
       </c>
       <c r="B11" t="s">
         <v>88</v>
@@ -2116,7 +2384,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>137</v>
+        <v>153</v>
       </c>
       <c r="B12" t="s">
         <v>81</v>

</xml_diff>